<commit_message>
Tickets: multi-ticket belongs in the workbook, and imports land in Draft
Add panel reverted to one worker, one ticket. Column M takes several types
separated by a comma (the file already allows it - the dropdown never blocked
typed values); the TICKETS sheet carries per-ticket detail.

Every imported ticket lands in Draft and is published from the Draft tab.

Export now carries the prototype's own eight workers and their real IDs, so
the sheet and the screen can be read against each other.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026-08-31-construction-tickets-add-bulk/Employee_Upload_Template_round_trip.xlsx
+++ b/2026-08-31-construction-tickets-add-bulk/Employee_Upload_Template_round_trip.xlsx
@@ -294,9 +294,9 @@
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>Optional, and now only a shortcut. Pick one type from the dropdown and the employee gets a DRAFT ticket with nothing in it but the type.
-For real ticket data — number, issued, expiry, issuing body, state — use the TICKETS sheet instead. One row per ticket, so a worker can hold more than one.
-If an employee appears on the TICKETS sheet, this cell is ignored for that employee.</t>
+        <t>Optional. To add more than one ticket, type the ticket types separated by a comma - the same way this workbook already handles Employee Payroll Allowance and Form Numbers. The dropdown is there to get the spelling right.
+Each type listed here creates a DRAFT ticket carrying nothing but the type.
+For the ticket's number, issued date, expiry, issuing body and state, use the TICKETS sheet instead - one row per ticket. If an employee appears on the TICKETS sheet, this cell is ignored for that employee.</t>
       </text>
     </comment>
   </commentList>
@@ -311,9 +311,9 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>LOCKED — do not edit.
+        <t>LOCKED - do not edit.
 Present only on an export that included existing tickets. A row that comes back with a Ticket Record ID updates that exact ticket. Blank creates a new one.
-This is what stops a re-upload duplicating everything.</t>
+EVERY ticket created by an import lands in DRAFT, in the Draft tab on the Construction Tickets page, and is published from there once it has been checked. An import never publishes straight into the live register.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -330,8 +330,9 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Required. Pick from the dropdown.
-A type that is not in the list is held back at review, where you can choose to add it to Manage Ticket Types. Types are never created silently.</t>
+        <t>Required. Pick from the dropdown, or type it.
+A type that is not in the list is held back at review, where you can choose to add it to Manage Ticket Types. Types are never created silently.
+One row per ticket, so a worker can hold as many as they hold - repeat their Employee ID on as many rows as you need.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -665,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -759,29 +760,37 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>EMP-0001</t>
+          <t>WKR-0001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>James</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Baker</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Cookie's Civil Pty</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Dump Truck Operator</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>VAR-1</t>
+          <t>EMP-1041</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>james@gmail.com</t>
+          <t>bk@cookiescivil.com.au</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -789,86 +798,399 @@
           <t>+61435265342</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Plant Equipment Operator (RIIWHS201D)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>EMP-0002</t>
+          <t>WKR-0002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ford</t>
+          <t>Dave</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Humphries</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
+          <t>Nguyen</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Cookie's Civil Pty</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Excavator Operator</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>VAR-2</t>
+          <t>EMP-1042</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>ford@hotmail.com</t>
+          <t>dave.n@cookiescivil.com.au</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>+61435265342</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="n"/>
+          <t>+61435265343</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>White Card (CPCCWHS1001), Forklift (LF)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>EMP-0003</t>
+          <t>WKR-0003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Matilda Grace</t>
+          <t>Jack</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Anderson</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
+          <t>Mercer</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Cookie's Civil Pty</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Pipelayer</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>VAR-3</t>
+          <t>EMP-1044</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>matilda@gmail.com</t>
+          <t>jack.m@cookiescivil.com.au</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>+61432145668</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="n"/>
+          <t>+61435265344</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="N4" s="2" t="n"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>WKR-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Whitcombe</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Varicon Info</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Leading Hand</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>EMP-1007</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>sam.w@varicon.com.au</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>+61435265345</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>WKR-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ellie</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Doust</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Varicon Info</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Foreman</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>EMP-1009</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ellie.d@varicon.com.au</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>+61435265346</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>WKR-0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Priya</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Raman</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Varicon Info</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Site Engineer</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>EMP-1012</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>priya.r@varicon.com.au</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>+61435265347</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>WKR-0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tui</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fa'alogo</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Northline Traffic</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Traffic Controller</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>EMP-2203</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>tui@northlinetraffic.com.au</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>+61435265348</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Subcontractor</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>WKR-0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Bianchi</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Northline Traffic</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Roller Operator</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>EMP-2210</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>marco@northlinetraffic.com.au</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>+61435265349</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Subcontractor</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="6">
@@ -1210,7 +1532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1291,42 +1613,40 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VAR-1</t>
+          <t>EMP-1041</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>James Baker</t>
+          <t>B K</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>White Card (CPCCWHS1001)</t>
+          <t>Plant Equipment Operator (RIIWHS201D)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0012 4471</t>
+          <t>532534</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>02/02/2021</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>SafeWork NSW</t>
-        </is>
-      </c>
+          <t>24/08/2023</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NSW</t>
-        </is>
-      </c>
+          <t>NT</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Not required</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1654,12 @@
       <c r="A3" s="5" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>VAR-1</t>
+          <t>EMP-1041</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>James Baker</t>
+          <t>B K</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1372,74 +1692,78 @@
           <t>NSW</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>VAR-2</t>
+          <t>EMP-1042</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Ford Humphries</t>
+          <t>Dave Nguyen</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Plant Equipment Operator (RIIWHS201D)</t>
+          <t>White Card (CPCCWHS1001)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>532534</t>
+          <t>0012 4471</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>24/08/2023</t>
+          <t>02/02/2021</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SafeWork NSW</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>NT</t>
-        </is>
-      </c>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>VAR-3</t>
+          <t>EMP-1044</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Matilda Grace Anderson</t>
+          <t>Jack Mercer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Forklift (LF)</t>
+          <t>White Card (CPCCWHS1001)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>4471223</t>
+          <t>0018 9902</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>19/07/2021</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>19/07/2026</t>
-        </is>
-      </c>
+          <t>08/11/2022</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>SafeWork NSW</t>
@@ -1450,12 +1774,94 @@
           <t>NSW</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Renewal booked</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EMP-2203</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Tui Fa'alogo</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Traffic Control (RIIWHS302E)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TM-7781</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>03/03/2029</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Aust. Traffic Svcs</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EMP-2210</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Marco Bianchi</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Plant Equipment Operator (RIIWHS201D)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>661201</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>11/05/2024</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>NT</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Roller only</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Tickets: one export, full ticket detail per row, and duplicate handling
Drops the template menu - the export always comes down filled with employees
and their current tickets. Every ticket row carries the add panel's full field
set, not just the type.

A ticket is identified by Ticket Record ID, else worker + type + number. Same
file twice is idempotent; a hand-added row updates rather than duplicating;
identical rows collapse; same type with a different number is a renewal and
both are kept. Review gained an Already on record count.

Also repairs two rules left behind by the reverted multi-type panel.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026-08-31-construction-tickets-add-bulk/Employee_Upload_Template_round_trip.xlsx
+++ b/2026-08-31-construction-tickets-add-bulk/Employee_Upload_Template_round_trip.xlsx
@@ -312,8 +312,10 @@
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <t>LOCKED - do not edit.
-Present only on an export that included existing tickets. A row that comes back with a Ticket Record ID updates that exact ticket. Blank creates a new one.
-EVERY ticket created by an import lands in DRAFT, in the Draft tab on the Construction Tickets page, and is published from there once it has been checked. An import never publishes straight into the live register.</t>
+This is the ticket's identity. A row that comes back with a Ticket Record ID updates that exact ticket. A row with it blank creates a new one.
+YOU CANNOT DOUBLE UP A TICKET. Where this cell is blank we match on Employee ID + Ticket Type + Ticket Number instead. A row matching an existing ticket on those three updates it, so uploading the same file twice changes nothing the second time, and adding a row by hand instead of editing the exported one does not create a copy.
+Same ticket type with a DIFFERENT number is a renewal, not a duplicate: both are kept and the older one is marked superseded.
+Every ticket an import creates lands in DRAFT and is published from the Draft tab on the Construction Tickets page.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -337,7 +339,8 @@
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>The number printed on the card. Text format — leading zeros matter.</t>
+        <t>The number printed on the card. Text format - leading zeros matter.
+Where Ticket Record ID is blank this is part of how we recognise the ticket, together with Employee ID and Ticket Type. Two rows with all three the same are one ticket, and are collapsed. Two rows with a different number here are two tickets - a renewal.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
@@ -978,7 +981,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1031,7 +1033,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1084,7 +1085,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1137,7 +1137,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1190,7 +1189,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="6">
@@ -1636,14 +1634,11 @@
           <t>24/08/2023</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>NT</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Not required</t>
@@ -1692,7 +1687,6 @@
           <t>NSW</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
@@ -1722,7 +1716,6 @@
           <t>02/02/2021</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>SafeWork NSW</t>
@@ -1733,7 +1726,6 @@
           <t>NSW</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
@@ -1763,7 +1755,6 @@
           <t>08/11/2022</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>SafeWork NSW</t>
@@ -1774,7 +1765,6 @@
           <t>NSW</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -1819,7 +1809,6 @@
           <t>NSW</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
@@ -1849,8 +1838,6 @@
           <t>11/05/2024</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>NT</t>

</xml_diff>

<commit_message>
Tickets: workers not employees, payment type filter, project picker
Active workers only, per Alec - calling a subcontractor an employee is a
characterisation we do not want in writing. Prototype language is worker
throughout; the workbook keeps its EMPLOYEES sheet and Employee ID column
because renaming a live importer column breaks saved copies. Flagged.

Include subcontractor workers replaced by a Payment type filter
(Subcontractor / Casual / Salary / Wages). Selecting a project now actually
offers a project. Live count under the filters.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026-08-31-construction-tickets-add-bulk/Employee_Upload_Template_round_trip.xlsx
+++ b/2026-08-31-construction-tickets-add-bulk/Employee_Upload_Template_round_trip.xlsx
@@ -261,9 +261,9 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>It is a pre-registered in the system. 
-It is optional. 
-Should be text format</t>
+        <t>It is pre-registered in the system. Optional. Should be text format.
+Salary, Wages, Casual or Subcontractor.
+NOTE: the product calls this a PAYMENT TYPE, not an employment type - and calls these people workers, not employees. The column name here is left as production has it so that saved copies of this workbook keep working; aligning the two is a deliberate decision, not a quiet edit.</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
@@ -919,7 +919,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Wages</t>
+          <t>Casual</t>
         </is>
       </c>
       <c r="K4" s="2" t="n"/>

</xml_diff>

<commit_message>
Tickets: one place for a ticket - drop the Tickets column from the export
Keeping column M gave the workbook two places to enter a ticket and a
precedence rule instead of an answer. The TICKETS sheet is now the only
place; the column is deleted from the EMPLOYEES sheet, its data validation
dropped and the remaining five dropdowns repointed after the column shift.

Files already saved with a Tickets column still import - deprecating what we
hand out is a different decision from dropping support.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026-08-31-construction-tickets-add-bulk/Employee_Upload_Template_round_trip.xlsx
+++ b/2026-08-31-construction-tickets-add-bulk/Employee_Upload_Template_round_trip.xlsx
@@ -290,13 +290,6 @@
       <text>
         <t>Form Numbers is optional. 
  should be separated by a comma</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. To add more than one ticket, type the ticket types separated by a comma - the same way this workbook already handles Employee Payroll Allowance and Form Numbers. The dropdown is there to get the spelling right.
-Each type listed here creates a DRAFT ticket carrying nothing but the type.
-For the ticket's number, issued date, expiry, issuing body and state, use the TICKETS sheet instead - one row per ticket. If an employee appears on the TICKETS sheet, this cell is ignored for that employee.</t>
       </text>
     </comment>
   </commentList>
@@ -669,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -754,11 +747,6 @@
           <t>Form Numbers</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
-        <is>
-          <t>Tickets</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -812,11 +800,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Plant Equipment Operator (RIIWHS201D)</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -870,11 +853,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>White Card (CPCCWHS1001), Forklift (LF)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -928,7 +906,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1191,7 +1168,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_EmploymentType!$A$1:$A$4</formula1>
     </dataValidation>
@@ -1206,9 +1183,6 @@
     </dataValidation>
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_CompanyName!$A$1:$A$187</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_Tickets!$A$1:$A$8</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>